<commit_message>
implement robust plate validation and persistent database storage with a real-time web dashboard
</commit_message>
<xml_diff>
--- a/detected_plates_2026-04-29.xlsx
+++ b/detected_plates_2026-04-29.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E16"/>
+  <dimension ref="A1:G12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -454,16 +454,26 @@
           <t>Category</t>
         </is>
       </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Duration</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>{7</t>
+          <t>A:1.71</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>{7</t>
+          <t>A:1.71</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -473,24 +483,34 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-04-29 22:47:24</t>
+          <t>2026-04-29 23:01:39</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
           <t>visitor</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Entered</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Active</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>AR Y 4A 7177</t>
+          <t>HK JO4A 1777</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>AR Y 4A 7177</t>
+          <t>HK JO4A 1777</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -500,51 +520,71 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>2026-04-29 22:47:25</t>
+          <t>2026-04-29 23:01:40</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
           <t>visitor</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Entered</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Active</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>;4 [ 777</t>
+          <t>HR 98 AA 7777</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>;4 [ 777</t>
+          <t>HR 98 AA 7777</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Aiden</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>2026-04-29 22:47:26</t>
+          <t>2026-04-29 23:01:41</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>visitor</t>
+          <t>teacher</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Entered</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Active</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>461117</t>
+          <t>HR Y8 44 7777</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>461117</t>
+          <t>HR Y8 44 7777</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -554,78 +594,108 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>2026-04-29 22:47:27</t>
+          <t>2026-04-29 23:03:26</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
           <t>visitor</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Entered</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Active</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>4; 1711</t>
+          <t>HR 98 AA 7777</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>4; 1711</t>
+          <t>HR 98 AA 7777</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Aiden</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>2026-04-29 22:47:27</t>
+          <t>2026-04-29 23:03:27</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>visitor</t>
+          <t>teacher</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Exited</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>0:01:46</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>AR YK A4 7777</t>
+          <t>HR 98 AA 7777</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>AR YK A4 7777</t>
+          <t>HR 98 AA 7777</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Aiden</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>2026-04-29 22:47:28</t>
+          <t>2026-04-29 23:03:28</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>visitor</t>
+          <t>teacher</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Entered</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Active</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>HR YX AA 7777</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>HR YX AA 7777</t>
+          <t>7</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -635,24 +705,34 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>2026-04-29 22:47:29</t>
+          <t>2026-04-29 23:04:24</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
           <t>visitor</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Entered</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Active</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>AR JO 4A 7777</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>AR JO 4A 7777</t>
+          <t>4</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -662,24 +742,34 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>2026-04-29 22:47:30</t>
+          <t>2026-04-29 23:04:29</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
           <t>visitor</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Entered</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>Active</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>HR :46 44 1177</t>
+          <t>P</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>HR :46 44 1177</t>
+          <t>P</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -689,24 +779,34 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>2026-04-29 22:47:30</t>
+          <t>2026-04-29 23:06:53</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
           <t>visitor</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Entered</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>Active</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>HR 98 AA 1777</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>HR 98 AA 1777</t>
+          <t>3</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -716,24 +816,34 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>2026-04-29 22:47:31</t>
+          <t>2026-04-29 23:07:03</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
           <t>visitor</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Entered</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>Active</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>HR 4+ ,A 7777</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>HR 4+ ,A 7777</t>
+          <t>4</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -743,7 +853,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>2026-04-29 22:47:32</t>
+          <t>2026-04-29 23:07:06</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -751,112 +861,14 @@
           <t>visitor</t>
         </is>
       </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>HR 98 AA 7777</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>HR 98 AA 7777</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>Aiden</t>
-        </is>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>2026-04-29 22:47:37</t>
-        </is>
-      </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>teacher</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>'"O% 1.</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>'"O% 1.</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>2026-04-29 22:48:02</t>
-        </is>
-      </c>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>visitor</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>;'117</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>;'117</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>2026-04-29 22:48:37</t>
-        </is>
-      </c>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>visitor</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>AK</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>AK</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>2026-04-29 22:48:38</t>
-        </is>
-      </c>
-      <c r="E16" t="inlineStr">
-        <is>
-          <t>visitor</t>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Exited</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>0:02:36</t>
         </is>
       </c>
     </row>

</xml_diff>